<commit_message>
added executable app and an installer for the user
</commit_message>
<xml_diff>
--- a/print/ar_template.xlsx
+++ b/print/ar_template.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Brant\PycharmProjects\AR-System\print\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{170E51D3-AB74-4FA3-AFBC-3BE28AA0554E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{862A7927-D39B-4E09-96E2-EB38DA8DD3D5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{5D05ADBB-1EBF-42F5-A7E4-14DE5F681420}"/>
   </bookViews>
@@ -269,14 +269,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="45">
+  <cellXfs count="44">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
@@ -791,458 +790,458 @@
       <c r="K1" s="2"/>
     </row>
     <row r="2" spans="1:18" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="6"/>
-      <c r="E2" s="29" t="s">
+      <c r="A2" s="5"/>
+      <c r="E2" s="28" t="s">
         <v>0</v>
       </c>
-      <c r="F2" s="29"/>
-      <c r="G2" s="29"/>
-      <c r="H2" s="29"/>
-      <c r="I2" s="29"/>
+      <c r="F2" s="28"/>
+      <c r="G2" s="28"/>
+      <c r="H2" s="28"/>
+      <c r="I2" s="28"/>
       <c r="K2" s="3"/>
-      <c r="L2" s="43" t="s">
+      <c r="L2" s="42" t="s">
         <v>3</v>
       </c>
-      <c r="M2" s="43"/>
-      <c r="N2" s="43"/>
-      <c r="O2" s="43"/>
-      <c r="P2" s="43"/>
-      <c r="Q2" s="16"/>
-      <c r="R2" s="15"/>
+      <c r="M2" s="42"/>
+      <c r="N2" s="42"/>
+      <c r="O2" s="42"/>
+      <c r="P2" s="42"/>
+      <c r="Q2" s="15"/>
+      <c r="R2" s="14"/>
     </row>
     <row r="3" spans="1:18" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="6"/>
-      <c r="E3" s="30" t="s">
+      <c r="A3" s="5"/>
+      <c r="E3" s="29" t="s">
         <v>1</v>
       </c>
-      <c r="F3" s="30"/>
-      <c r="G3" s="30"/>
-      <c r="H3" s="30"/>
-      <c r="I3" s="30"/>
-      <c r="J3" s="30"/>
+      <c r="F3" s="29"/>
+      <c r="G3" s="29"/>
+      <c r="H3" s="29"/>
+      <c r="I3" s="29"/>
+      <c r="J3" s="29"/>
       <c r="K3" s="3"/>
-      <c r="L3" s="44"/>
-      <c r="M3" s="44"/>
-      <c r="N3" s="44"/>
-      <c r="O3" s="44"/>
-      <c r="P3" s="44"/>
-      <c r="Q3" s="17"/>
-      <c r="R3" s="15"/>
+      <c r="L3" s="43"/>
+      <c r="M3" s="43"/>
+      <c r="N3" s="43"/>
+      <c r="O3" s="43"/>
+      <c r="P3" s="43"/>
+      <c r="Q3" s="16"/>
+      <c r="R3" s="14"/>
     </row>
     <row r="4" spans="1:18" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="6"/>
-      <c r="E4" s="30" t="s">
+      <c r="A4" s="5"/>
+      <c r="E4" s="29" t="s">
         <v>16</v>
       </c>
-      <c r="F4" s="30"/>
-      <c r="G4" s="30"/>
-      <c r="H4" s="30"/>
-      <c r="I4" s="30"/>
-      <c r="J4" s="30"/>
+      <c r="F4" s="29"/>
+      <c r="G4" s="29"/>
+      <c r="H4" s="29"/>
+      <c r="I4" s="29"/>
+      <c r="J4" s="29"/>
       <c r="K4" s="3"/>
-      <c r="L4" s="34" t="s">
+      <c r="L4" s="33" t="s">
         <v>4</v>
       </c>
-      <c r="M4" s="35"/>
-      <c r="N4" s="35"/>
-      <c r="O4" s="35"/>
+      <c r="M4" s="34"/>
+      <c r="N4" s="34"/>
+      <c r="O4" s="34"/>
       <c r="P4" s="3"/>
-      <c r="Q4" s="18"/>
+      <c r="Q4" s="17"/>
     </row>
     <row r="5" spans="1:18" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="6"/>
-      <c r="E5" s="30" t="s">
+      <c r="A5" s="5"/>
+      <c r="E5" s="29" t="s">
         <v>2</v>
       </c>
-      <c r="F5" s="30"/>
-      <c r="G5" s="30"/>
-      <c r="H5" s="30"/>
-      <c r="I5" s="30"/>
-      <c r="J5" s="30"/>
+      <c r="F5" s="29"/>
+      <c r="G5" s="29"/>
+      <c r="H5" s="29"/>
+      <c r="I5" s="29"/>
+      <c r="J5" s="29"/>
       <c r="K5" s="3"/>
-      <c r="L5" s="34"/>
-      <c r="M5" s="35"/>
-      <c r="N5" s="35"/>
-      <c r="O5" s="35"/>
+      <c r="L5" s="33"/>
+      <c r="M5" s="34"/>
+      <c r="N5" s="34"/>
+      <c r="O5" s="34"/>
       <c r="P5" s="3"/>
-      <c r="Q5" s="18"/>
+      <c r="Q5" s="17"/>
     </row>
     <row r="6" spans="1:18" ht="5.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="6"/>
-      <c r="Q6" s="6"/>
+      <c r="A6" s="5"/>
+      <c r="Q6" s="5"/>
     </row>
     <row r="7" spans="1:18" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="6"/>
-      <c r="B7" s="10" t="s">
+      <c r="A7" s="5"/>
+      <c r="B7" s="9" t="s">
         <v>5</v>
       </c>
-      <c r="C7" s="33"/>
-      <c r="D7" s="33"/>
-      <c r="E7" s="33"/>
-      <c r="F7" s="33"/>
-      <c r="G7" s="4"/>
-      <c r="H7" s="4"/>
-      <c r="I7" s="4"/>
-      <c r="J7" s="4"/>
-      <c r="K7" s="4"/>
-      <c r="L7" s="4"/>
-      <c r="M7" s="4"/>
-      <c r="N7" s="10" t="s">
+      <c r="C7" s="32"/>
+      <c r="D7" s="32"/>
+      <c r="E7" s="32"/>
+      <c r="F7" s="32"/>
+      <c r="G7" s="32"/>
+      <c r="H7" s="32"/>
+      <c r="I7" s="32"/>
+      <c r="J7" s="32"/>
+      <c r="K7" s="32"/>
+      <c r="L7" s="32"/>
+      <c r="M7" s="32"/>
+      <c r="N7" s="9" t="s">
         <v>6</v>
       </c>
-      <c r="O7" s="19"/>
-      <c r="P7" s="5"/>
-      <c r="Q7" s="7"/>
-    </row>
-    <row r="8" spans="1:18" s="14" customFormat="1" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="11"/>
-      <c r="B8" s="12" t="s">
+      <c r="O7" s="18"/>
+      <c r="P7" s="4"/>
+      <c r="Q7" s="6"/>
+    </row>
+    <row r="8" spans="1:18" s="13" customFormat="1" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="10"/>
+      <c r="B8" s="11" t="s">
         <v>9</v>
       </c>
-      <c r="C8" s="37" t="s">
+      <c r="C8" s="36" t="s">
         <v>7</v>
       </c>
-      <c r="D8" s="37"/>
-      <c r="E8" s="37"/>
-      <c r="F8" s="37" t="s">
+      <c r="D8" s="36"/>
+      <c r="E8" s="36"/>
+      <c r="F8" s="36" t="s">
         <v>8</v>
       </c>
-      <c r="G8" s="37"/>
-      <c r="H8" s="37"/>
-      <c r="I8" s="10" t="s">
+      <c r="G8" s="36"/>
+      <c r="H8" s="36"/>
+      <c r="I8" s="9" t="s">
         <v>10</v>
       </c>
-      <c r="J8" s="10"/>
-      <c r="K8" s="10" t="s">
+      <c r="J8" s="9"/>
+      <c r="K8" s="9" t="s">
         <v>11</v>
       </c>
-      <c r="L8" s="10"/>
-      <c r="M8" s="10"/>
-      <c r="N8" s="10"/>
-      <c r="O8" s="10"/>
-      <c r="P8" s="10"/>
-      <c r="Q8" s="13"/>
+      <c r="L8" s="9"/>
+      <c r="M8" s="9"/>
+      <c r="N8" s="9"/>
+      <c r="O8" s="9"/>
+      <c r="P8" s="9"/>
+      <c r="Q8" s="12"/>
     </row>
     <row r="9" spans="1:18" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="6"/>
-      <c r="B9" s="24"/>
-      <c r="C9" s="24"/>
-      <c r="D9" s="24"/>
-      <c r="E9" s="24"/>
-      <c r="F9" s="25"/>
-      <c r="G9" s="25"/>
-      <c r="H9" s="25"/>
-      <c r="I9" s="24"/>
-      <c r="J9" s="24"/>
-      <c r="K9" s="24"/>
-      <c r="L9" s="24"/>
-      <c r="M9" s="24"/>
-      <c r="N9" s="24"/>
-      <c r="O9" s="24"/>
-      <c r="P9" s="24"/>
-      <c r="Q9" s="6"/>
+      <c r="A9" s="5"/>
+      <c r="B9" s="23"/>
+      <c r="C9" s="23"/>
+      <c r="D9" s="23"/>
+      <c r="E9" s="23"/>
+      <c r="F9" s="24"/>
+      <c r="G9" s="24"/>
+      <c r="H9" s="24"/>
+      <c r="I9" s="23"/>
+      <c r="J9" s="23"/>
+      <c r="K9" s="23"/>
+      <c r="L9" s="23"/>
+      <c r="M9" s="23"/>
+      <c r="N9" s="23"/>
+      <c r="O9" s="23"/>
+      <c r="P9" s="23"/>
+      <c r="Q9" s="5"/>
     </row>
     <row r="10" spans="1:18" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="6"/>
-      <c r="B10" s="24"/>
-      <c r="C10" s="24"/>
-      <c r="D10" s="24"/>
-      <c r="E10" s="24"/>
-      <c r="F10" s="24"/>
-      <c r="H10" s="24"/>
-      <c r="I10" s="24"/>
-      <c r="J10" s="24"/>
-      <c r="K10" s="24"/>
-      <c r="L10" s="24"/>
-      <c r="M10" s="24"/>
-      <c r="N10" s="24"/>
-      <c r="O10" s="24"/>
-      <c r="P10" s="24"/>
-      <c r="Q10" s="6"/>
+      <c r="A10" s="5"/>
+      <c r="B10" s="23"/>
+      <c r="C10" s="23"/>
+      <c r="D10" s="23"/>
+      <c r="E10" s="23"/>
+      <c r="F10" s="23"/>
+      <c r="H10" s="23"/>
+      <c r="I10" s="23"/>
+      <c r="J10" s="23"/>
+      <c r="K10" s="23"/>
+      <c r="L10" s="23"/>
+      <c r="M10" s="23"/>
+      <c r="N10" s="23"/>
+      <c r="O10" s="23"/>
+      <c r="P10" s="23"/>
+      <c r="Q10" s="5"/>
     </row>
     <row r="11" spans="1:18" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="6"/>
-      <c r="B11" s="24"/>
-      <c r="C11" s="24"/>
-      <c r="D11" s="24"/>
-      <c r="E11" s="24"/>
-      <c r="F11" s="24"/>
-      <c r="G11" s="24"/>
-      <c r="H11" s="24"/>
-      <c r="I11" s="24"/>
-      <c r="J11" s="24"/>
-      <c r="K11" s="24"/>
-      <c r="L11" s="24"/>
-      <c r="M11" s="24"/>
-      <c r="N11" s="24"/>
-      <c r="O11" s="24"/>
-      <c r="P11" s="24"/>
-      <c r="Q11" s="6"/>
+      <c r="A11" s="5"/>
+      <c r="B11" s="23"/>
+      <c r="C11" s="23"/>
+      <c r="D11" s="23"/>
+      <c r="E11" s="23"/>
+      <c r="F11" s="23"/>
+      <c r="G11" s="23"/>
+      <c r="H11" s="23"/>
+      <c r="I11" s="23"/>
+      <c r="J11" s="23"/>
+      <c r="K11" s="23"/>
+      <c r="L11" s="23"/>
+      <c r="M11" s="23"/>
+      <c r="N11" s="23"/>
+      <c r="O11" s="23"/>
+      <c r="P11" s="23"/>
+      <c r="Q11" s="5"/>
     </row>
     <row r="12" spans="1:18" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="6"/>
-      <c r="B12" s="24"/>
-      <c r="C12" s="24"/>
-      <c r="D12" s="24"/>
-      <c r="E12" s="24"/>
-      <c r="F12" s="24"/>
-      <c r="G12" s="24"/>
-      <c r="H12" s="24"/>
-      <c r="I12" s="24"/>
-      <c r="J12" s="24"/>
-      <c r="K12" s="24"/>
-      <c r="L12" s="24"/>
-      <c r="M12" s="24"/>
-      <c r="N12" s="24"/>
-      <c r="O12" s="24"/>
-      <c r="P12" s="24"/>
-      <c r="Q12" s="6"/>
+      <c r="A12" s="5"/>
+      <c r="B12" s="23"/>
+      <c r="C12" s="23"/>
+      <c r="D12" s="23"/>
+      <c r="E12" s="23"/>
+      <c r="F12" s="23"/>
+      <c r="G12" s="23"/>
+      <c r="H12" s="23"/>
+      <c r="I12" s="23"/>
+      <c r="J12" s="23"/>
+      <c r="K12" s="23"/>
+      <c r="L12" s="23"/>
+      <c r="M12" s="23"/>
+      <c r="N12" s="23"/>
+      <c r="O12" s="23"/>
+      <c r="P12" s="23"/>
+      <c r="Q12" s="5"/>
     </row>
     <row r="13" spans="1:18" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="6"/>
-      <c r="B13" s="24"/>
-      <c r="C13" s="24"/>
-      <c r="D13" s="24"/>
-      <c r="E13" s="24"/>
-      <c r="F13" s="24"/>
-      <c r="G13" s="24"/>
-      <c r="H13" s="24"/>
-      <c r="I13" s="24"/>
-      <c r="J13" s="24"/>
-      <c r="K13" s="24"/>
-      <c r="L13" s="24"/>
-      <c r="M13" s="24"/>
-      <c r="N13" s="24"/>
-      <c r="O13" s="24"/>
-      <c r="P13" s="24"/>
-      <c r="Q13" s="6"/>
+      <c r="A13" s="5"/>
+      <c r="B13" s="23"/>
+      <c r="C13" s="23"/>
+      <c r="D13" s="23"/>
+      <c r="E13" s="23"/>
+      <c r="F13" s="23"/>
+      <c r="G13" s="23"/>
+      <c r="H13" s="23"/>
+      <c r="I13" s="23"/>
+      <c r="J13" s="23"/>
+      <c r="K13" s="23"/>
+      <c r="L13" s="23"/>
+      <c r="M13" s="23"/>
+      <c r="N13" s="23"/>
+      <c r="O13" s="23"/>
+      <c r="P13" s="23"/>
+      <c r="Q13" s="5"/>
     </row>
     <row r="14" spans="1:18" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="6"/>
-      <c r="B14" s="24"/>
-      <c r="C14" s="24"/>
-      <c r="D14" s="24"/>
-      <c r="E14" s="24"/>
-      <c r="F14" s="24"/>
-      <c r="G14" s="24"/>
-      <c r="H14" s="24"/>
-      <c r="I14" s="24"/>
-      <c r="J14" s="24"/>
-      <c r="K14" s="24"/>
-      <c r="L14" s="24"/>
-      <c r="M14" s="24"/>
-      <c r="N14" s="24"/>
-      <c r="O14" s="24"/>
-      <c r="P14" s="24"/>
-      <c r="Q14" s="6"/>
+      <c r="A14" s="5"/>
+      <c r="B14" s="23"/>
+      <c r="C14" s="23"/>
+      <c r="D14" s="23"/>
+      <c r="E14" s="23"/>
+      <c r="F14" s="23"/>
+      <c r="G14" s="23"/>
+      <c r="H14" s="23"/>
+      <c r="I14" s="23"/>
+      <c r="J14" s="23"/>
+      <c r="K14" s="23"/>
+      <c r="L14" s="23"/>
+      <c r="M14" s="23"/>
+      <c r="N14" s="23"/>
+      <c r="O14" s="23"/>
+      <c r="P14" s="23"/>
+      <c r="Q14" s="5"/>
     </row>
     <row r="15" spans="1:18" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="6"/>
-      <c r="B15" s="24"/>
-      <c r="C15" s="24"/>
-      <c r="D15" s="24"/>
-      <c r="E15" s="24"/>
-      <c r="F15" s="24"/>
-      <c r="G15" s="24"/>
-      <c r="H15" s="24"/>
-      <c r="I15" s="24"/>
-      <c r="J15" s="24"/>
-      <c r="K15" s="24"/>
-      <c r="L15" s="24"/>
-      <c r="M15" s="24"/>
-      <c r="N15" s="24"/>
-      <c r="O15" s="24"/>
-      <c r="P15" s="24"/>
-      <c r="Q15" s="6"/>
+      <c r="A15" s="5"/>
+      <c r="B15" s="23"/>
+      <c r="C15" s="23"/>
+      <c r="D15" s="23"/>
+      <c r="E15" s="23"/>
+      <c r="F15" s="23"/>
+      <c r="G15" s="23"/>
+      <c r="H15" s="23"/>
+      <c r="I15" s="23"/>
+      <c r="J15" s="23"/>
+      <c r="K15" s="23"/>
+      <c r="L15" s="23"/>
+      <c r="M15" s="23"/>
+      <c r="N15" s="23"/>
+      <c r="O15" s="23"/>
+      <c r="P15" s="23"/>
+      <c r="Q15" s="5"/>
     </row>
     <row r="16" spans="1:18" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="6"/>
-      <c r="B16" s="24"/>
-      <c r="C16" s="24"/>
-      <c r="D16" s="24"/>
-      <c r="E16" s="24"/>
-      <c r="F16" s="24"/>
-      <c r="G16" s="24"/>
-      <c r="H16" s="24"/>
-      <c r="I16" s="24"/>
-      <c r="J16" s="24"/>
-      <c r="K16" s="24"/>
-      <c r="L16" s="24"/>
-      <c r="M16" s="24"/>
-      <c r="N16" s="24"/>
-      <c r="O16" s="24"/>
-      <c r="P16" s="24"/>
-      <c r="Q16" s="6"/>
+      <c r="A16" s="5"/>
+      <c r="B16" s="23"/>
+      <c r="C16" s="23"/>
+      <c r="D16" s="23"/>
+      <c r="E16" s="23"/>
+      <c r="F16" s="23"/>
+      <c r="G16" s="23"/>
+      <c r="H16" s="23"/>
+      <c r="I16" s="23"/>
+      <c r="J16" s="23"/>
+      <c r="K16" s="23"/>
+      <c r="L16" s="23"/>
+      <c r="M16" s="23"/>
+      <c r="N16" s="23"/>
+      <c r="O16" s="23"/>
+      <c r="P16" s="23"/>
+      <c r="Q16" s="5"/>
     </row>
     <row r="17" spans="1:17" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="6"/>
-      <c r="B17" s="24"/>
-      <c r="C17" s="24"/>
-      <c r="D17" s="24"/>
-      <c r="E17" s="24"/>
-      <c r="F17" s="24"/>
-      <c r="G17" s="24"/>
-      <c r="H17" s="24"/>
-      <c r="I17" s="24"/>
-      <c r="J17" s="24"/>
-      <c r="K17" s="24"/>
-      <c r="L17" s="24"/>
-      <c r="M17" s="24"/>
-      <c r="N17" s="24"/>
-      <c r="O17" s="24"/>
-      <c r="P17" s="24"/>
-      <c r="Q17" s="6"/>
+      <c r="A17" s="5"/>
+      <c r="B17" s="23"/>
+      <c r="C17" s="23"/>
+      <c r="D17" s="23"/>
+      <c r="E17" s="23"/>
+      <c r="F17" s="23"/>
+      <c r="G17" s="23"/>
+      <c r="H17" s="23"/>
+      <c r="I17" s="23"/>
+      <c r="J17" s="23"/>
+      <c r="K17" s="23"/>
+      <c r="L17" s="23"/>
+      <c r="M17" s="23"/>
+      <c r="N17" s="23"/>
+      <c r="O17" s="23"/>
+      <c r="P17" s="23"/>
+      <c r="Q17" s="5"/>
     </row>
     <row r="18" spans="1:17" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="6"/>
-      <c r="B18" s="24"/>
-      <c r="C18" s="24"/>
-      <c r="D18" s="24"/>
-      <c r="E18" s="24"/>
-      <c r="F18" s="24"/>
-      <c r="G18" s="24"/>
-      <c r="H18" s="24"/>
-      <c r="I18" s="24"/>
-      <c r="J18" s="24"/>
-      <c r="K18" s="24"/>
-      <c r="L18" s="24"/>
-      <c r="M18" s="24"/>
-      <c r="N18" s="24"/>
-      <c r="O18" s="24"/>
-      <c r="P18" s="24"/>
-      <c r="Q18" s="6"/>
+      <c r="A18" s="5"/>
+      <c r="B18" s="23"/>
+      <c r="C18" s="23"/>
+      <c r="D18" s="23"/>
+      <c r="E18" s="23"/>
+      <c r="F18" s="23"/>
+      <c r="G18" s="23"/>
+      <c r="H18" s="23"/>
+      <c r="I18" s="23"/>
+      <c r="J18" s="23"/>
+      <c r="K18" s="23"/>
+      <c r="L18" s="23"/>
+      <c r="M18" s="23"/>
+      <c r="N18" s="23"/>
+      <c r="O18" s="23"/>
+      <c r="P18" s="23"/>
+      <c r="Q18" s="5"/>
     </row>
     <row r="19" spans="1:17" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="6"/>
-      <c r="B19" s="24"/>
-      <c r="C19" s="24"/>
-      <c r="D19" s="24"/>
-      <c r="E19" s="24"/>
-      <c r="F19" s="24"/>
-      <c r="G19" s="24"/>
-      <c r="H19" s="24"/>
-      <c r="I19" s="24"/>
-      <c r="J19" s="24"/>
-      <c r="K19" s="24"/>
-      <c r="L19" s="24"/>
-      <c r="M19" s="24"/>
-      <c r="N19" s="24"/>
-      <c r="O19" s="24"/>
-      <c r="P19" s="24"/>
-      <c r="Q19" s="6"/>
+      <c r="A19" s="5"/>
+      <c r="B19" s="23"/>
+      <c r="C19" s="23"/>
+      <c r="D19" s="23"/>
+      <c r="E19" s="23"/>
+      <c r="F19" s="23"/>
+      <c r="G19" s="23"/>
+      <c r="H19" s="23"/>
+      <c r="I19" s="23"/>
+      <c r="J19" s="23"/>
+      <c r="K19" s="23"/>
+      <c r="L19" s="23"/>
+      <c r="M19" s="23"/>
+      <c r="N19" s="23"/>
+      <c r="O19" s="23"/>
+      <c r="P19" s="23"/>
+      <c r="Q19" s="5"/>
     </row>
     <row r="20" spans="1:17" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="6"/>
-      <c r="B20" s="24"/>
-      <c r="C20" s="24"/>
-      <c r="D20" s="24"/>
-      <c r="E20" s="24"/>
-      <c r="F20" s="24"/>
-      <c r="G20" s="24"/>
-      <c r="H20" s="24"/>
-      <c r="I20" s="24"/>
-      <c r="J20" s="24"/>
-      <c r="K20" s="24"/>
-      <c r="L20" s="24"/>
-      <c r="M20" s="24"/>
-      <c r="N20" s="24"/>
-      <c r="O20" s="24"/>
-      <c r="P20" s="24"/>
-      <c r="Q20" s="6"/>
+      <c r="A20" s="5"/>
+      <c r="B20" s="23"/>
+      <c r="C20" s="23"/>
+      <c r="D20" s="23"/>
+      <c r="E20" s="23"/>
+      <c r="F20" s="23"/>
+      <c r="G20" s="23"/>
+      <c r="H20" s="23"/>
+      <c r="I20" s="23"/>
+      <c r="J20" s="23"/>
+      <c r="K20" s="23"/>
+      <c r="L20" s="23"/>
+      <c r="M20" s="23"/>
+      <c r="N20" s="23"/>
+      <c r="O20" s="23"/>
+      <c r="P20" s="23"/>
+      <c r="Q20" s="5"/>
     </row>
     <row r="21" spans="1:17" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B21" s="26"/>
-      <c r="C21" s="27"/>
-      <c r="D21" s="27"/>
-      <c r="E21" s="27"/>
-      <c r="F21" s="27"/>
-      <c r="G21" s="27"/>
-      <c r="H21" s="27"/>
-      <c r="I21" s="27"/>
-      <c r="J21" s="28"/>
-      <c r="K21" s="28"/>
-      <c r="L21" s="28"/>
-      <c r="M21" s="28"/>
-      <c r="N21" s="28"/>
-      <c r="O21" s="28"/>
-      <c r="P21" s="28"/>
-      <c r="Q21" s="9"/>
+      <c r="B21" s="25"/>
+      <c r="C21" s="26"/>
+      <c r="D21" s="26"/>
+      <c r="E21" s="26"/>
+      <c r="F21" s="26"/>
+      <c r="G21" s="26"/>
+      <c r="H21" s="26"/>
+      <c r="I21" s="26"/>
+      <c r="J21" s="27"/>
+      <c r="K21" s="27"/>
+      <c r="L21" s="27"/>
+      <c r="M21" s="27"/>
+      <c r="N21" s="27"/>
+      <c r="O21" s="27"/>
+      <c r="P21" s="27"/>
+      <c r="Q21" s="8"/>
     </row>
     <row r="22" spans="1:17" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B22" s="38" t="s">
+      <c r="B22" s="37" t="s">
         <v>12</v>
       </c>
-      <c r="C22" s="39"/>
-      <c r="D22" s="39"/>
-      <c r="E22" s="39"/>
-      <c r="F22" s="39"/>
-      <c r="G22" s="39"/>
-      <c r="H22" s="39"/>
-      <c r="I22" s="22"/>
-      <c r="J22" s="21"/>
-      <c r="K22" s="14"/>
-      <c r="L22" s="14"/>
-      <c r="M22" s="14"/>
-      <c r="N22" s="14"/>
-      <c r="O22" s="14"/>
-      <c r="P22" s="14"/>
-      <c r="Q22" s="11"/>
+      <c r="C22" s="38"/>
+      <c r="D22" s="38"/>
+      <c r="E22" s="38"/>
+      <c r="F22" s="38"/>
+      <c r="G22" s="38"/>
+      <c r="H22" s="38"/>
+      <c r="I22" s="21"/>
+      <c r="J22" s="20"/>
+      <c r="K22" s="13"/>
+      <c r="L22" s="13"/>
+      <c r="M22" s="13"/>
+      <c r="N22" s="13"/>
+      <c r="O22" s="13"/>
+      <c r="P22" s="13"/>
+      <c r="Q22" s="10"/>
     </row>
     <row r="23" spans="1:17" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B23" s="38"/>
-      <c r="C23" s="39"/>
-      <c r="D23" s="39"/>
-      <c r="E23" s="39"/>
-      <c r="F23" s="39"/>
-      <c r="G23" s="39"/>
-      <c r="H23" s="39"/>
-      <c r="J23" s="36" t="s">
+      <c r="B23" s="37"/>
+      <c r="C23" s="38"/>
+      <c r="D23" s="38"/>
+      <c r="E23" s="38"/>
+      <c r="F23" s="38"/>
+      <c r="G23" s="38"/>
+      <c r="H23" s="38"/>
+      <c r="J23" s="35" t="s">
         <v>14</v>
       </c>
-      <c r="K23" s="14"/>
-      <c r="L23" s="14"/>
-      <c r="M23" s="14"/>
-      <c r="N23" s="14"/>
-      <c r="O23" s="14"/>
-      <c r="P23" s="14"/>
-      <c r="Q23" s="11"/>
+      <c r="K23" s="13"/>
+      <c r="L23" s="13"/>
+      <c r="M23" s="13"/>
+      <c r="N23" s="13"/>
+      <c r="O23" s="13"/>
+      <c r="P23" s="13"/>
+      <c r="Q23" s="10"/>
     </row>
     <row r="24" spans="1:17" ht="7.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B24" s="40" t="s">
+      <c r="B24" s="39" t="s">
         <v>13</v>
       </c>
-      <c r="C24" s="41"/>
-      <c r="D24" s="42"/>
-      <c r="E24" s="42"/>
-      <c r="F24" s="42"/>
-      <c r="J24" s="36"/>
-      <c r="K24" s="23"/>
-      <c r="L24" s="23"/>
-      <c r="M24" s="23"/>
-      <c r="N24" s="23"/>
-      <c r="O24" s="23"/>
-      <c r="P24" s="23"/>
-      <c r="Q24" s="11"/>
+      <c r="C24" s="40"/>
+      <c r="D24" s="41"/>
+      <c r="E24" s="41"/>
+      <c r="F24" s="41"/>
+      <c r="J24" s="35"/>
+      <c r="K24" s="22"/>
+      <c r="L24" s="22"/>
+      <c r="M24" s="22"/>
+      <c r="N24" s="22"/>
+      <c r="O24" s="22"/>
+      <c r="P24" s="22"/>
+      <c r="Q24" s="10"/>
     </row>
     <row r="25" spans="1:17" ht="10.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B25" s="40"/>
-      <c r="C25" s="41"/>
-      <c r="D25" s="42"/>
-      <c r="E25" s="42"/>
-      <c r="F25" s="42"/>
-      <c r="J25" s="20"/>
-      <c r="K25" s="31" t="s">
+      <c r="B25" s="39"/>
+      <c r="C25" s="40"/>
+      <c r="D25" s="41"/>
+      <c r="E25" s="41"/>
+      <c r="F25" s="41"/>
+      <c r="J25" s="19"/>
+      <c r="K25" s="30" t="s">
         <v>15</v>
       </c>
-      <c r="L25" s="31"/>
-      <c r="M25" s="31"/>
-      <c r="N25" s="31"/>
-      <c r="O25" s="31"/>
-      <c r="P25" s="31"/>
-      <c r="Q25" s="32"/>
+      <c r="L25" s="30"/>
+      <c r="M25" s="30"/>
+      <c r="N25" s="30"/>
+      <c r="O25" s="30"/>
+      <c r="P25" s="30"/>
+      <c r="Q25" s="31"/>
     </row>
     <row r="26" spans="1:17" ht="4.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B26" s="8"/>
+      <c r="B26" s="7"/>
       <c r="C26" s="2"/>
       <c r="D26" s="2"/>
       <c r="E26" s="2"/>
@@ -1250,14 +1249,14 @@
       <c r="G26" s="2"/>
       <c r="H26" s="2"/>
       <c r="I26" s="2"/>
-      <c r="J26" s="8"/>
+      <c r="J26" s="7"/>
       <c r="K26" s="2"/>
       <c r="L26" s="2"/>
       <c r="M26" s="2"/>
       <c r="N26" s="2"/>
       <c r="O26" s="2"/>
       <c r="P26" s="2"/>
-      <c r="Q26" s="9"/>
+      <c r="Q26" s="8"/>
     </row>
     <row r="27" spans="1:17" ht="7.5" customHeight="1" x14ac:dyDescent="0.25"/>
   </sheetData>
@@ -1267,7 +1266,6 @@
     <mergeCell ref="E4:J4"/>
     <mergeCell ref="E5:J5"/>
     <mergeCell ref="K25:Q25"/>
-    <mergeCell ref="C7:F7"/>
     <mergeCell ref="L4:L5"/>
     <mergeCell ref="M4:O5"/>
     <mergeCell ref="J23:J24"/>
@@ -1277,6 +1275,7 @@
     <mergeCell ref="D24:F25"/>
     <mergeCell ref="L2:P3"/>
     <mergeCell ref="F8:H8"/>
+    <mergeCell ref="C7:M7"/>
   </mergeCells>
   <pageMargins left="0" right="0" top="0" bottom="0" header="0" footer="0"/>
   <pageSetup paperSize="10003" fitToWidth="0" orientation="portrait" horizontalDpi="0" verticalDpi="0" r:id="rId1"/>

</xml_diff>

<commit_message>
updated the prod color to also display centered in the print preview
</commit_message>
<xml_diff>
--- a/print/ar_template.xlsx
+++ b/print/ar_template.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Brant\PycharmProjects\AR-System\print\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{862A7927-D39B-4E09-96E2-EB38DA8DD3D5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{18BFDDC3-E5FF-4B1C-8B89-3E32A37B9308}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{5D05ADBB-1EBF-42F5-A7E4-14DE5F681420}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="17">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="18">
   <si>
     <t>MASTERBATCH PHILIPPINES INC.</t>
   </si>
@@ -90,6 +90,9 @@
   </si>
   <si>
     <t>Telephone No.: (02) 7002-3720  | Contact No.: 0908-8106546</t>
+  </si>
+  <si>
+    <t>das</t>
   </si>
 </sst>
 </file>
@@ -269,7 +272,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="44">
+  <cellXfs count="45">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
@@ -318,8 +321,11 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
+      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
@@ -330,9 +336,6 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -364,6 +367,9 @@
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
@@ -396,7 +402,7 @@
       <xdr:col>3</xdr:col>
       <xdr:colOff>125556</xdr:colOff>
       <xdr:row>4</xdr:row>
-      <xdr:rowOff>90363</xdr:rowOff>
+      <xdr:rowOff>60597</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -764,8 +770,9 @@
     <col min="5" max="5" width="3.42578125" style="1" customWidth="1"/>
     <col min="6" max="6" width="13.7109375" style="1" customWidth="1"/>
     <col min="7" max="7" width="9.140625" style="1"/>
-    <col min="8" max="9" width="6.85546875" style="1" customWidth="1"/>
-    <col min="10" max="10" width="12.28515625" style="1" customWidth="1"/>
+    <col min="8" max="8" width="9.85546875" style="1" customWidth="1"/>
+    <col min="9" max="9" width="3.140625" style="1" customWidth="1"/>
+    <col min="10" max="10" width="13.28515625" style="1" customWidth="1"/>
     <col min="11" max="11" width="6.42578125" style="1" customWidth="1"/>
     <col min="12" max="12" width="7" style="1" customWidth="1"/>
     <col min="13" max="13" width="3.5703125" style="1" customWidth="1"/>
@@ -789,15 +796,15 @@
       <c r="J1" s="2"/>
       <c r="K1" s="2"/>
     </row>
-    <row r="2" spans="1:18" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="5"/>
-      <c r="E2" s="28" t="s">
+      <c r="E2" s="29" t="s">
         <v>0</v>
       </c>
-      <c r="F2" s="28"/>
-      <c r="G2" s="28"/>
-      <c r="H2" s="28"/>
-      <c r="I2" s="28"/>
+      <c r="F2" s="29"/>
+      <c r="G2" s="29"/>
+      <c r="H2" s="29"/>
+      <c r="I2" s="29"/>
       <c r="K2" s="3"/>
       <c r="L2" s="42" t="s">
         <v>3</v>
@@ -809,16 +816,16 @@
       <c r="Q2" s="15"/>
       <c r="R2" s="14"/>
     </row>
-    <row r="3" spans="1:18" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:18" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="5"/>
-      <c r="E3" s="29" t="s">
+      <c r="E3" s="30" t="s">
         <v>1</v>
       </c>
-      <c r="F3" s="29"/>
-      <c r="G3" s="29"/>
-      <c r="H3" s="29"/>
-      <c r="I3" s="29"/>
-      <c r="J3" s="29"/>
+      <c r="F3" s="30"/>
+      <c r="G3" s="30"/>
+      <c r="H3" s="30"/>
+      <c r="I3" s="30"/>
+      <c r="J3" s="30"/>
       <c r="K3" s="3"/>
       <c r="L3" s="43"/>
       <c r="M3" s="43"/>
@@ -828,16 +835,16 @@
       <c r="Q3" s="16"/>
       <c r="R3" s="14"/>
     </row>
-    <row r="4" spans="1:18" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:18" ht="9.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="5"/>
-      <c r="E4" s="29" t="s">
+      <c r="E4" s="30" t="s">
         <v>16</v>
       </c>
-      <c r="F4" s="29"/>
-      <c r="G4" s="29"/>
-      <c r="H4" s="29"/>
-      <c r="I4" s="29"/>
-      <c r="J4" s="29"/>
+      <c r="F4" s="30"/>
+      <c r="G4" s="30"/>
+      <c r="H4" s="30"/>
+      <c r="I4" s="30"/>
+      <c r="J4" s="30"/>
       <c r="K4" s="3"/>
       <c r="L4" s="33" t="s">
         <v>4</v>
@@ -850,14 +857,14 @@
     </row>
     <row r="5" spans="1:18" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="5"/>
-      <c r="E5" s="29" t="s">
+      <c r="E5" s="30" t="s">
         <v>2</v>
       </c>
-      <c r="F5" s="29"/>
-      <c r="G5" s="29"/>
-      <c r="H5" s="29"/>
-      <c r="I5" s="29"/>
-      <c r="J5" s="29"/>
+      <c r="F5" s="30"/>
+      <c r="G5" s="30"/>
+      <c r="H5" s="30"/>
+      <c r="I5" s="30"/>
+      <c r="J5" s="30"/>
       <c r="K5" s="3"/>
       <c r="L5" s="33"/>
       <c r="M5" s="34"/>
@@ -866,26 +873,28 @@
       <c r="P5" s="3"/>
       <c r="Q5" s="17"/>
     </row>
-    <row r="6" spans="1:18" ht="5.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:18" ht="4.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="5"/>
       <c r="Q6" s="5"/>
     </row>
-    <row r="7" spans="1:18" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:18" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="5"/>
-      <c r="B7" s="9" t="s">
+      <c r="B7" s="28" t="s">
         <v>5</v>
       </c>
-      <c r="C7" s="32"/>
-      <c r="D7" s="32"/>
-      <c r="E7" s="32"/>
-      <c r="F7" s="32"/>
-      <c r="G7" s="32"/>
-      <c r="H7" s="32"/>
-      <c r="I7" s="32"/>
-      <c r="J7" s="32"/>
-      <c r="K7" s="32"/>
-      <c r="L7" s="32"/>
-      <c r="M7" s="32"/>
+      <c r="C7" s="44" t="s">
+        <v>17</v>
+      </c>
+      <c r="D7" s="44"/>
+      <c r="E7" s="44"/>
+      <c r="F7" s="44"/>
+      <c r="G7" s="44"/>
+      <c r="H7" s="44"/>
+      <c r="I7" s="44"/>
+      <c r="J7" s="44"/>
+      <c r="K7" s="44"/>
+      <c r="L7" s="44"/>
+      <c r="M7" s="44"/>
       <c r="N7" s="9" t="s">
         <v>6</v>
       </c>
@@ -908,10 +917,10 @@
       </c>
       <c r="G8" s="36"/>
       <c r="H8" s="36"/>
-      <c r="I8" s="9" t="s">
+      <c r="I8" s="36" t="s">
         <v>10</v>
       </c>
-      <c r="J8" s="9"/>
+      <c r="J8" s="36"/>
       <c r="K8" s="9" t="s">
         <v>11</v>
       </c>
@@ -1230,15 +1239,15 @@
       <c r="E25" s="41"/>
       <c r="F25" s="41"/>
       <c r="J25" s="19"/>
-      <c r="K25" s="30" t="s">
+      <c r="K25" s="31" t="s">
         <v>15</v>
       </c>
-      <c r="L25" s="30"/>
-      <c r="M25" s="30"/>
-      <c r="N25" s="30"/>
-      <c r="O25" s="30"/>
-      <c r="P25" s="30"/>
-      <c r="Q25" s="31"/>
+      <c r="L25" s="31"/>
+      <c r="M25" s="31"/>
+      <c r="N25" s="31"/>
+      <c r="O25" s="31"/>
+      <c r="P25" s="31"/>
+      <c r="Q25" s="32"/>
     </row>
     <row r="26" spans="1:17" ht="4.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B26" s="7"/>
@@ -1260,7 +1269,7 @@
     </row>
     <row r="27" spans="1:17" ht="7.5" customHeight="1" x14ac:dyDescent="0.25"/>
   </sheetData>
-  <mergeCells count="15">
+  <mergeCells count="16">
     <mergeCell ref="E2:I2"/>
     <mergeCell ref="E3:J3"/>
     <mergeCell ref="E4:J4"/>
@@ -1276,6 +1285,7 @@
     <mergeCell ref="L2:P3"/>
     <mergeCell ref="F8:H8"/>
     <mergeCell ref="C7:M7"/>
+    <mergeCell ref="I8:J8"/>
   </mergeCells>
   <pageMargins left="0" right="0" top="0" bottom="0" header="0" footer="0"/>
   <pageSetup paperSize="10003" fitToWidth="0" orientation="portrait" horizontalDpi="0" verticalDpi="0" r:id="rId1"/>

</xml_diff>